<commit_message>
updated BCEU, BCRBQ, BPMCCS, BFPAT, BFPIaE, NBPoNVP, SYVBT
</commit_message>
<xml_diff>
--- a/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
+++ b/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
@@ -9839,14 +9839,18 @@
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="688c5d3b-a76a-458b-b159-91c2a1154680">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
-    <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010027350D42B0D95040ACC873ED5DCB146E" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07e9ea90ad522b71e445466745b665d9">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="688c5d3b-a76a-458b-b159-91c2a1154680" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2528a4ec313a4f0a1f4e92f7a0496c8f" ns2:_="">
+    <xsd:import namespace="688c5d3b-a76a-458b-b159-91c2a1154680"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -9857,6 +9861,11 @@
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -9864,7 +9873,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="79748b23-d81a-423e-9112-21109dc864e6" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="688c5d3b-a76a-458b-b159-91c2a1154680" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -9886,6 +9895,33 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="eca5b831-c3dc-41cf-bd85-218b82cecb21" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -10005,19 +10041,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6055987-FA8E-4520-AD86-240857E14832}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35C3175E-805B-45C6-81AE-F5D1F1603BB9}"/>
 </file>
</xml_diff>